<commit_message>
Translate headlines to German and update datasets
Update preprocessing/headline_extract.ipynb to translate headlines to German (GoogleTranslator target set to 'de'), rename translated column to Headline_GER, and adjust ordered_columns accordingly. Cleaned notebook outputs/execution counts. Regenerated binary Excel outputs preprocessing/headlines_dataset.xlsx and preprocessing/headlines_dataset_15sample.xlsx to reflect the changes.
</commit_message>
<xml_diff>
--- a/preprocessing/headlines_dataset_15sample.xlsx
+++ b/preprocessing/headlines_dataset_15sample.xlsx
@@ -424,7 +424,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>Headline_EN</t>
+          <t>Headline_GER</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
@@ -511,7 +511,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Ex-Sailor Pardoned By Trump Says He’s SUING Obama And Comey</t>
+          <t>Von Trump begnadigter Ex-Seemann sagt, er verklage Obama und Comey</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -542,7 +542,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Broward County Election Supervisor Brenda Snipes Resigns Amid Florida Voter Fraud</t>
+          <t>Brenda Snipes, Wahlleiterin im Broward County, tritt wegen Wahlbetrugs in Florida zurück</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -573,7 +573,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>I'll Say What Kavanaugh Wouldn't: Christine Ford Was Part Of The Political Hit On Him &amp; Here's The Audio Evidence</t>
+          <t>Ich sage, was Kavanaugh nicht sagen würde: Christine Ford war Teil des politischen Anschlags auf ihn und hier ist der Audiobeweis</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -604,7 +604,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Uranium One Bombshell: Evidence of Bribery, Extortion, Kickbacks, Money Laundering, and More!</t>
+          <t>Uranium One Bombshell: Beweise für Bestechung, Erpressung, Schmiergelder, Geldwäsche und mehr!</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -635,7 +635,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Sore Loser: Stacey Abrams Ends Challenges In Georgia Gubernatorial Race - Won't Concede - Set To File Lawsuit</t>
+          <t>Schlechter Verlierer: Stacey Abrams beendet Herausforderungen im Rennen um den Gouverneursposten in Georgia – wird nicht zugeben – will Klage einreichen</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -666,7 +666,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Local Police &amp; Feds Impose INFORMATION BLACKOUT in Las Vegas Shooting</t>
+          <t>Lokale Polizei und Fed verhängen Informationssperre bei Schießerei in Las Vegas</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -697,7 +697,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>German cardinal: liturgical ‘blessing’ for gay unions is ‘truly…sacrilegious’</t>
+          <t>Deutscher Kardinal: Liturgischer „Segen“ für Schwulengemeinschaften ist „wirklich … Sakrileg“</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -728,7 +728,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Court orders White House to restore CNN correspondent Jim Acosta’s press credential</t>
+          <t>Das Gericht ordnet an, dass das Weiße Haus die Presseberechtigung des CNN-Korrespondenten Jim Acosta wiederherstellen muss</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -759,7 +759,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>After Calling for Guns &amp; Ammo Confiscation &amp; Universal Gun Registration, the American Medical Association Should Think About Taking "American" Out of Their Name</t>
+          <t>Nachdem die American Medical Association die Beschlagnahmung von Waffen und Munition sowie die allgemeine Waffenregistrierung gefordert hat, sollte sie darüber nachdenken, „amerikanisch“ aus ihrem Namen zu streichen</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -790,7 +790,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Has Trump Opened the Door?</t>
+          <t>Hat Trump die Tür geöffnet?</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -821,7 +821,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Judge Orders White House To Restore Jim Acosta' Press Pass - Trump Responds</t>
+          <t>Richter befiehlt dem Weißen Haus, den Presseausweis von Jim Acosta wiederherzustellen – Trump antwortet</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -852,7 +852,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>DOJ Surrenders: 3D Print Gun Files Are Protected Under First Amendment</t>
+          <t>DOJ kapituliert: 3D-Druck-Waffenakten sind durch den ersten Verfassungszusatz geschützt</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -883,7 +883,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>U.S. warns of 'sonic attacks' in China</t>
+          <t>Die USA warnen vor „Schallangriffen“ in China</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -914,7 +914,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>US bloggers banned from entering UK</t>
+          <t>US-Bloggern wurde die Einreise nach Großbritannien verboten</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -945,7 +945,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>RICHARD LITTLEJOHN: The capital sees its first stabbings of the year</t>
+          <t>RICHARD LITTLEJOHN: In der Hauptstadt kommt es zum ersten Mal in diesem Jahr zu Messerstechereien</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -976,7 +976,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Foolish Religion Author Gary Wills: ‘The Religion of the Qur’an Is a Religion of Peace’</t>
+          <t>Gary Wills, Autor der törichten Religion: „Die Religion des Korans ist eine Religion des Friedens“</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -1007,7 +1007,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Mueller Report: 'US Forced EU to Follow Through on Sanctions Without Proof'</t>
+          <t>Mueller-Bericht: „Die USA haben die EU gezwungen, ihre Sanktionen ohne Beweise durchzusetzen“</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -1038,7 +1038,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Derbyshire Cheers For Hard Brexit | Blog Posts</t>
+          <t>Derbyshire jubelt über harten Brexit | Blogbeiträge</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -1069,7 +1069,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>SPECIAL REPORT: Pope Francis Accused of Inaction in Notorious Sex Abuse Cases</t>
+          <t>SONDERBERICHT: Papst Franziskus wird Untätigkeit in Fällen berüchtigten sexuellen Missbrauchs vorgeworfen</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -1100,7 +1100,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Illegal alien wanted for attempted murder in NC arrested at US-Mexico border</t>
+          <t>Illegaler Ausländer, der wegen versuchten Mordes in North Carolina gesucht wird, an der Grenze zwischen den USA und Mexiko festgenommen</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -1131,7 +1131,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Man arrested for allegedly buying gun used in killing of Ohio officers at scene of 911 hang-up call</t>
+          <t>Mann wurde verhaftet, weil er am Tatort des 911-Auflegens angeblich eine Waffe gekauft hatte, mit der Polizisten aus Ohio getötet wurden</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -1162,7 +1162,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Student says anti-Semitism still an issue in McGill student government</t>
+          <t>Student sagt, Antisemitismus sei immer noch ein Problem in der McGill-Studentenregierung</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -1193,7 +1193,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Not So Fast</t>
+          <t>Nicht so schnell</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -1224,7 +1224,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>The Sun is getting cooler and dimmer, but scientists aren’t worried</t>
+          <t>Die Sonne wird kühler und schwächer, aber die Wissenschaftler machen sich keine Sorgen</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -1255,7 +1255,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>It’s Airborne: Officials Warn That The “Black Death” Plague Could Spread Rapidly</t>
+          <t>Es ist in der Luft: Beamte warnen, dass sich die Seuche „Schwarzer Tod“ schnell ausbreiten könnte</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -1286,7 +1286,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Humanity’s WIPEOUT Foreshadowed? World Health Chief: Global Pandemic Imminent</t>
+          <t>Ist die Auslöschung der Menschheit vorhersehbar? Weltgesundheitschef: Globale Pandemie steht unmittelbar bevor</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -1317,7 +1317,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Mueller Report Being Reviewed By A.G. Barr On Saturday</t>
+          <t>Mueller-Bericht wird am Samstag von A.G. Barr geprüft</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -1348,7 +1348,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Hundreds of Priests Accused in Pennsylvania, Church of Accompaniment in Crisis</t>
+          <t>Hunderte Priester in Pennsylvania angeklagt, Begleitkirche in der Krise</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -1379,7 +1379,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>The Never-Trumpers Are Never Coming Back</t>
+          <t>Die Never-Trumpers kommen niemals zurück</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -1410,7 +1410,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Clinton Email IG Report Rips FBI, Comey, &amp; Lynch… Plus A Whole Lot More!</t>
+          <t>Clintons E-Mail-IG-Bericht zerreißt FBI, Comey und Lynch … und noch viel mehr!</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
@@ -1441,7 +1441,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>ICE arrests 20 in Kansas City during 4-day operation targeting criminal aliens</t>
+          <t>ICE verhaftet 20 Personen in Kansas City während einer viertägigen Operation gegen kriminelle Ausländer</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
@@ -1503,7 +1503,7 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>﻿Vatican Theologian Sacked for Questioning “Merciful” Pope’s Pontificate</t>
+          <t>﻿Vatikanischer Theologe entlassen, weil er das Pontifikat des „barmherzigen“ Papstes in Frage gestellt hat</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
@@ -1534,7 +1534,7 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Police training up for deployment to NI in case of no-deal Brexit</t>
+          <t>Die Polizei bereitet sich auf den Einsatz in Nordirland für den Fall eines No-Deal-Brexit vor</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
@@ -1565,7 +1565,7 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Understanding Mueller: What you need to know about the report on the Russia probe</t>
+          <t>Mueller verstehen: Was Sie über den Bericht zur Russland-Untersuchung wissen müssen</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
@@ -1596,7 +1596,7 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Texas: Cop Walks Into Home She Thought Was Hers, Kills Innocent Homeowner—Not Arrested</t>
+          <t>Texas: Polizist betritt das Haus, von dem sie dachte, es gehöre ihr, und tötet einen unschuldigen Hausbesitzer – wird aber nicht verhaftet</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
@@ -1627,7 +1627,7 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Democrat’s Friend Louis Farrakhan In Iran: “Death to America!” – America Is The “Great Satan”</t>
+          <t>Demokratenfreund Louis Farrakhan im Iran: „Tod für Amerika!“ – Amerika ist der „große Satan“</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
@@ -1658,7 +1658,7 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>America's Immigration Voice.</t>
+          <t>Amerikas Einwanderungsstimme.</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
@@ -1689,7 +1689,7 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>The Mueller Report Finally Drops, Dems Prepare List of Demands</t>
+          <t>Der Mueller-Bericht wird endlich fallen gelassen, die Demokraten bereiten eine Liste mit Forderungen vor</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
@@ -1720,7 +1720,7 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Lawmaker makes shocking claim about the Vegas massacre (video)</t>
+          <t>Gesetzgeber macht schockierende Behauptung zum Massaker in Las Vegas (Video)</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
@@ -1751,7 +1751,7 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Google colluded with Clinton campaign with ‘silent donations’</t>
+          <t>Google hat mit Clintons Wahlkampf mit „stillen Spenden“ zusammengearbeitet</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
@@ -1782,7 +1782,7 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Roger Stone associate Jerome Corsi celebrates end of Mueller probe after REFUSING to sign plea deal</t>
+          <t>Jerome Corsi, Mitarbeiter von Roger Stone, feiert das Ende der Mueller-Untersuchung, nachdem er sich geweigert hat, einen Plädoyervertrag zu unterzeichnen</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
@@ -1813,7 +1813,7 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Asteroid Will Skim By Earth Days Before Christmas: It Is ‘Potentially Hazardous’</t>
+          <t>Asteroid wird wenige Tage vor Weihnachten an der Erde vorbeifliegen: Er ist „potenziell gefährlich“</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
@@ -1844,7 +1844,7 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Trump Advisers Upbeat: Mueller ‘Doesn’t Have the Goods’</t>
+          <t>Trump-Berater optimistisch: Mueller „hat nicht das Zeug dazu“</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
@@ -1875,7 +1875,7 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Facebook Bans Outline to Stop Jihadi Attacks on Americans.</t>
+          <t>Facebook-Verbotsentwurf zur Verhinderung dschihadistischer Angriffe auf Amerikaner.</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
@@ -1906,7 +1906,7 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Bill Clinton: ‘I Did The Right Thing’ During Lewinsky Affair; ‘I Do Not’ Owe Her Apology</t>
+          <t>Bill Clinton: „Ich habe das Richtige getan“ während der Lewinsky-Affäre; „Ich schulde ihr keine Entschuldigung.“</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
@@ -1937,7 +1937,7 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>Beto O'Rourke says he still believes that Trump conspired with Russia</t>
+          <t>Beto O'Rourke sagt, er glaube immer noch, dass Trump mit Russland konspiriert habe</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
@@ -1968,7 +1968,7 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Robert Mueller III Rests His Case—Dems NEVER Will</t>
+          <t>Robert Mueller III lässt seinen Fall ruhen – die Demokraten werden es NIEMALS tun</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
@@ -1999,7 +1999,7 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>Who Is Behind the Internet Thought Police?</t>
+          <t>Wer steckt hinter der Internet-Gedankenpolizei?</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
@@ -2030,7 +2030,7 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>Hillary Cracks Racist Joke After Mixing Up Cory Booker &amp; Eric Holder: "They All Look The Same"</t>
+          <t>Hillary macht einen rassistischen Witz, nachdem sie Cory Booker und Eric Holder verwechselt hat: „Sie sehen alle gleich aus“</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
@@ -2061,7 +2061,7 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>Kavanaugh Nomination Is Exploding in Trump’s Face</t>
+          <t>Kavanaughs Nominierung explodiert vor Trumps Gesicht</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
@@ -2092,7 +2092,7 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>Brazilian arms dealer arrested in the United States</t>
+          <t>Brasilianischer Waffenhändler in den USA festgenommen</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
@@ -2123,7 +2123,7 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>Watch: Campus Commie Has Profanity-Laden Hissy Fit, Pours Beverage on FSU Republicans</t>
+          <t>Anschauen: Campus Commie hat einen mit Obszönitäten beladenen, zischenden Anfall und schüttet Getränke über FSU-Republikaner aus</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
@@ -2154,7 +2154,7 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>Mueller Is Done, but the Trump Investigations Are Just Heating Up</t>
+          <t>Mueller ist fertig, aber die Trump-Ermittlungen nehmen nur noch Fahrt auf</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
@@ -2185,7 +2185,7 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>Obama Judge Rules To Upend Georgia Election</t>
+          <t>Obama-Richter entscheidet, Wahl in Georgia zu ändern</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
@@ -2216,7 +2216,7 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>2020 Democrats Demand Mueller Report’s Public Release</t>
+          <t>Die Demokraten von 2020 fordern die Veröffentlichung des Mueller-Berichts</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
@@ -2247,7 +2247,7 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>Foreign Secretary Jeremy Hunt says the UK should not 'underestimate its strength' after Brexit</t>
+          <t>Außenminister Jeremy Hunt sagt, Großbritannien dürfe „seine Stärke“ nach dem Brexit nicht unterschätzen</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
@@ -2278,7 +2278,7 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>Beware sonic weapon attacks, US tells citizens in China</t>
+          <t>Hüten Sie sich vor Angriffen mit Schallwaffen, sagen die USA den Bürgern in China</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
@@ -2309,7 +2309,7 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>End The Korean War!</t>
+          <t>Beende den Koreakrieg!</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
@@ -2340,7 +2340,7 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>An Anti-Semitic Purge At McGill University</t>
+          <t>Eine antisemitische Säuberung an der McGill University</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
@@ -2371,7 +2371,7 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>3rd Highest Ranked Dem Civil Rights Hero Appeared w/Farrakhan, Won't Condemn</t>
+          <t>Dritthöchster demokratischer Bürgerrechtsheld erschien mit Farrakhan, wird nicht verurteilen</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
@@ -2402,7 +2402,7 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>Pope Francis: Ross Douthat &amp; Massimo Faggioli Debate Catholic Church’s Future</t>
+          <t>Papst Franziskus: Ross Douthat und Massimo Faggioli diskutieren über die Zukunft der katholischen Kirche</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
@@ -2433,7 +2433,7 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>Ex-Muslim Catholics to Pope Francis: “Naiveté in the face of Islam is suicidal and very dangerous”</t>
+          <t>Ehemalige muslimische Katholiken an Papst Franziskus: „Naivität gegenüber dem Islam ist selbstmörderisch und sehr gefährlich“</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
@@ -2464,7 +2464,7 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>Don Trump Jr uses Maury Povich paternity meme to mock Democrats</t>
+          <t>Don Trump Jr. nutzt das Vaterschafts-Mem von Maury Povich, um sich über die Demokraten lustig zu machen</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
@@ -2495,7 +2495,7 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>The Far Right Is Trying to Co-opt the Yellow Vests</t>
+          <t>Die extreme Rechte versucht, die Gelbwesten zu vereinnahmen</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
@@ -2526,7 +2526,7 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>The Eerie Silence</t>
+          <t>Die unheimliche Stille</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
@@ -2557,7 +2557,7 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>George III Lost America.</t>
+          <t>Georg III. hat Amerika verloren.</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
@@ -2588,7 +2588,7 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>Being Skeptical Of Documented Liars Attacking a Supreme Court Nominee Is A Good Thing - Here's Why</t>
+          <t>Skeptisch gegenüber dokumentierten Lügnern zu sein, die einen Kandidaten für den Obersten Gerichtshof angreifen, ist eine gute Sache – hier ist der Grund dafür</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
@@ -2619,7 +2619,7 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>Cardinal Müller: Blessing homosexual couples would be an ‘atrocity’</t>
+          <t>Kardinal Müller: Die Segnung homosexueller Paare wäre eine „Gräueltat“</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
@@ -2650,7 +2650,7 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>EU Profits From Trading With UK While London Loses Money – Political Campaigner</t>
+          <t>EU profitiert vom Handel mit Großbritannien, während London Geld verliert – politischer Aktivist</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
@@ -2681,7 +2681,7 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>Majority of Tory voters want their MPs to back Theresa May's deal</t>
+          <t>Die Mehrheit der Tory-Wähler möchte, dass ihre Abgeordneten den Deal von Theresa May unterstützen</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
@@ -2712,7 +2712,7 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>Pope Francis' sexual abuse commission, hit by resignations and criticism, gets a reboot</t>
+          <t>Die von Rücktritten und Kritik betroffene Kommission für sexuellen Missbrauch von Papst Franziskus erhält einen Neustart</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
@@ -2743,7 +2743,7 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>Ex-MI6 chief says Theresa May’s Brexit deal ‘threatens national security,’ hurts US relationship</t>
+          <t>Ex-MI6-Chef sagt, Theresa Mays Brexit-Deal „bedroht die nationale Sicherheit“ und schadet den Beziehungen zu den USA</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
@@ -2774,7 +2774,7 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>The American Jewish Historical Society Hosts Destroy Israel Event</t>
+          <t>Die American Jewish Historical Society veranstaltet die Veranstaltung „Zerstöre Israel“.</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
@@ -2805,7 +2805,7 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>Homeschooling Protects Children from Violence and Marxism</t>
+          <t>Homeschooling schützt Kinder vor Gewalt und Marxismus</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
@@ -2836,7 +2836,7 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>Receipt Shows Paddock Had Another Guest in His Room Before Shooting</t>
+          <t>Aus der Quittung geht hervor, dass Paddock vor den Dreharbeiten einen weiteren Gast in seinem Zimmer hatte</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
@@ -2867,7 +2867,7 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>US reacts to end of Mueller probe with relief, skepticism</t>
+          <t>Die USA reagieren mit Erleichterung und Skepsis auf das Ende der Mueller-Untersuchung</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
@@ -2898,7 +2898,7 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>Are Western spies supporting the new “Ukrainian White Helmets”?</t>
+          <t>Unterstützen westliche Spione die neuen „ukrainischen Weißhelme“?</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
@@ -2929,7 +2929,7 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>Between Vladimir Putin and the West, the standoff continues</t>
+          <t>Zwischen Wladimir Putin und dem Westen geht die Pattsituation weiter</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
@@ -2960,7 +2960,7 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>Francis, pope of the poor and ecology? Or pope of the global elite?</t>
+          <t>Franziskus, Papst der Armen und der Ökologie? Oder Papst der globalen Elite?</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
@@ -2991,7 +2991,7 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>Joe Biden and the G-7 want to spend billions of dollars to finance “green projects” in the Third World</t>
+          <t>Joe Biden und die G-7 wollen Milliarden von Dollar ausgeben, um „grüne Projekte“ in der Dritten Welt zu finanzieren</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
@@ -3022,7 +3022,7 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>Fight against homophobia: an “ambassador for LGBT+ rights” will be appointed “before the end of the year”, announces Elisabeth Borne</t>
+          <t>Kampf gegen Homophobie: Noch in diesem Jahr werde ein „Botschafter für LGBT+-Rechte“ ernannt, kündigt Elisabeth Borne an</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
@@ -3053,7 +3053,7 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>The Ministry of Defense of the Russian Federation published data on work with tick infections in biological laboratories of the United States in Ukraine</t>
+          <t>Das Verteidigungsministerium der Russischen Föderation veröffentlichte Daten über die Arbeit mit Zeckeninfektionen in biologischen Labors der Vereinigten Staaten in der Ukraine</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
@@ -3084,7 +3084,7 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>Ukraine – Russian missile targeting civilians accidentally kills several Ukrainian soldiers</t>
+          <t>Ukraine – Russische Rakete, die auf Zivilisten zielt, tötet versehentlich mehrere ukrainische Soldaten</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
@@ -3115,7 +3115,7 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>A “City COP” to fight climate change</t>
+          <t>Eine „City COP“ zur Bekämpfung des Klimawandels</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
@@ -3146,7 +3146,7 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>Biden calls MAGA ideology 'extreme'</t>
+          <t>Biden nennt MAGA-Ideologie „extrem“</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
@@ -3177,7 +3177,7 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>An exemplary sanction expertly studied by our fantastically intelligent leaders!!!</t>
+          <t>Eine beispielhafte Sanktion, die von unseren fantastisch intelligenten Führern fachmännisch untersucht wurde!!!</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
@@ -3208,7 +3208,7 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>A monstrous mountain of plastic is predicted for 2060</t>
+          <t>Für 2060 wird ein monströser Plastikberg vorhergesagt</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
@@ -3239,7 +3239,7 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>“The European Union's climate strategy is set to increase deforestation globally”</t>
+          <t>„Die Klimastrategie der Europäischen Union soll die Entwaldung weltweit verstärken“</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
@@ -3270,7 +3270,7 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>Macron wants to “piss off” the unvaccinated: a frightening totalitarian turn</t>
+          <t>Macron will die Ungeimpften „verärgern“: eine erschreckende totalitäre Wende</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
@@ -3301,7 +3301,7 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>WEF wants children to learn in the metaverse to fight climate change</t>
+          <t>Das WEF möchte, dass Kinder im Metaversum lernen, den Klimawandel zu bekämpfen</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
@@ -3332,7 +3332,7 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>Environmental fanaticism: latest news from Europe</t>
+          <t>Umweltfanatismus: Aktuelle Nachrichten aus Europa</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
@@ -3363,7 +3363,7 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>NATO and Russia pretend not to be afraid</t>
+          <t>Die NATO und Russland tun so, als hätten sie keine Angst</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
@@ -3394,7 +3394,7 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>Sustainable Olympism</t>
+          <t>Nachhaltiger Olympismus</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
@@ -3425,7 +3425,7 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>What if France offered asylum to Americans who want to have an abortion</t>
+          <t>Was wäre, wenn Frankreich Amerikanern, die eine Abtreibung wünschen, Asyl anbieten würde?</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
@@ -3456,7 +3456,7 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>Central banks do not control inflation</t>
+          <t>Zentralbanken kontrollieren die Inflation nicht</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
@@ -3487,7 +3487,7 @@
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>Climate – Researchers are developing an index 450 sunscreen</t>
+          <t>Klima – Forscher entwickeln einen Sonnenschutz mit Index 450</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
@@ -3518,7 +3518,7 @@
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>Another thirty years lost</t>
+          <t>Weitere dreißig Jahre verloren</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
@@ -3549,7 +3549,7 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>Faced with the lawless liar, Marine fought well</t>
+          <t>Angesichts des gesetzlosen Lügners kämpfte Marine gut</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
@@ -3580,7 +3580,7 @@
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>All of Emmanuel Macron's health policy decisions cost more than 600 billion, for what result?</t>
+          <t>Alle gesundheitspolitischen Entscheidungen von Emmanuel Macron haben mehr als 600 Milliarden gekostet, für welches Ergebnis?</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
@@ -3611,7 +3611,7 @@
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>The Minsk Agreements, what Minsk agreements?</t>
+          <t>Die Minsker Abkommen, welche Minsker Abkommen?</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
@@ -3642,7 +3642,7 @@
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>[Ukraine] Why is Russia not isolated from the rest of the world?</t>
+          <t>[Ukraine] Warum ist Russland nicht vom Rest der Welt isoliert?</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
@@ -3673,7 +3673,7 @@
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>Catastrophe and panic</t>
+          <t>Katastrophe und Panik</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
@@ -3704,7 +3704,7 @@
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>Russian state television reassures viewers about nuclear war: “We will all die one day”</t>
+          <t>Russisches Staatsfernsehen beruhigt Zuschauer vor Atomkrieg: „Eines Tages werden wir alle sterben“</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
@@ -3735,7 +3735,7 @@
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>Climate: France is poorly equipped to face future crises</t>
+          <t>Klima: Frankreich ist für künftige Krisen schlecht gerüstet</t>
         </is>
       </c>
       <c r="C106" t="inlineStr">
@@ -3766,7 +3766,7 @@
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>Vladimir Putin sends his army to the center of the Earth to “denazify the lava”</t>
+          <t>Wladimir Putin schickt seine Armee in den Mittelpunkt der Erde, um „die Lava zu entnazifizieren“</t>
         </is>
       </c>
       <c r="C107" t="inlineStr">
@@ -3797,7 +3797,7 @@
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>From Texas, Viktor Orban calls on American conservatives to “join forces” in the face of the “culture war” led by the left</t>
+          <t>Aus Texas fordert Viktor Orban die amerikanischen Konservativen auf, angesichts des von der Linken geführten „Kulturkrieges“ „ihre Kräfte zu bündeln“.</t>
         </is>
       </c>
       <c r="C108" t="inlineStr">
@@ -3828,7 +3828,7 @@
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>United States: Not everything is a national emergency</t>
+          <t>Vereinigte Staaten: Nicht alles ist ein nationaler Notfall</t>
         </is>
       </c>
       <c r="C109" t="inlineStr">
@@ -3859,7 +3859,7 @@
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>Taiwan: Xi Jinping tells Joe Biden not to “play with fire”</t>
+          <t>Taiwan: Xi Jinping fordert Joe Biden auf, nicht „mit dem Feuer zu spielen“</t>
         </is>
       </c>
       <c r="C110" t="inlineStr">
@@ -3890,7 +3890,7 @@
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>UN Commissioner Filippo Grandi points out double standards in the treatment of refugees</t>
+          <t>UN-Kommissar Filippo Grandi weist auf Doppelmoral bei Behandlung von Flüchtlingen hin</t>
         </is>
       </c>
       <c r="C111" t="inlineStr">
@@ -3921,7 +3921,7 @@
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>Secret NATO report via Wikileaks showed miserable Russian forces, urge for tactical nuclear weapons</t>
+          <t>Geheimer NATO-Bericht via Wikileaks zeigte miserable russische Streitkräfte, Drang zu taktischen Atomwaffen</t>
         </is>
       </c>
       <c r="C112" t="inlineStr">
@@ -3952,7 +3952,7 @@
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>Western sanctions have the opposite effect: Russia's energy revenues are higher than before the war</t>
+          <t>Westliche Sanktionen bewirken das Gegenteil: Rußlands Energie-Einnahmen höher als vor dem Krieg</t>
         </is>
       </c>
       <c r="C113" t="inlineStr">
@@ -3983,7 +3983,7 @@
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>The Ukrainian is using the war and the fascists to stay in power. Prize question: When was the last 8 p.m. daily news program without a report about Ukraine's President Zelenskyj - silly costumed in NATO olive, demanding weapons and money? “Zelenskyj” in the search field on tagesschau.de results in more than 1,400 hits for the last three months. Tagesschau.de lists Zelensky videos more than 500 times: hero worship for a remote-controlled tyrant who prolongs the state of war to consolidate his own position and sacrifices hundreds of lives every day to achieve this. On the other hand, the Tagesschau failed to mention the globally respected advice of former US Secretary of State Henry Kissinger that Zelensky should voluntarily cede territory to Russia and make peace in order to avoid a pan-European catastrophe. Kissinger's realism obviously didn't fit into the propaganda stuff for the ARD-aktuell editorial team, which was loyal to the green line.</t>
+          <t>Der Ukrainer nutzt den Krieg und die Faschisten, um sich an der Macht zu halten. Preisfrage: Wann lief die letzte 20-Uhr-Tagesschau ohne Beitrag über Ukraines Präsidenten Selenskyj – albern kostümiert in NATO-Oliv, Waffen und Geld fordernd? „Selenskyj“ im Suchfeld auf tagesschau.de ergibt für die letzten drei Monate mehr als 1 400 Treffer. Tagesschau.de listet darunter mehr als 500-mal Selenskyj-Videos: Heldenverehrung für einen ferngesteuerten Gewaltherrscher, der den Kriegszustand zur Festigung der eigenen Position verlängert und dafür täglich hunderte Menschenleben opfert. Hingegen verschwieg die Tagesschau den weltweit beachteten Rat des einstigen US-Außenministers Henry Kissinger, Selenskyj solle zur Vermeidung einer gesamteuropäischen Katastrophe freiwillig Territorium an Russland abtreten und Frieden schließen. Kissingers Realismus passte der giftgrün-linientreuen ARD-aktuell-Redaktion ersichtlich nicht in den Propagandakram.</t>
         </is>
       </c>
       <c r="C114" t="inlineStr">
@@ -4014,7 +4014,7 @@
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>Survey reveals: 83 percent of Germans want better border protection</t>
+          <t>Umfrage deckt auf: 83 Prozent der Deutschen wünschen sich besseren Grenzschutz</t>
         </is>
       </c>
       <c r="C115" t="inlineStr">
@@ -4045,7 +4045,7 @@
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>Up to $380 per barrel: Experts warn of dramatic increases in oil prices</t>
+          <t>Bis 380 US-Dollar pro Barrel: Experten warnen von dramatischen Erdölpreissteigerungen</t>
         </is>
       </c>
       <c r="C116" t="inlineStr">
@@ -4076,7 +4076,7 @@
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>Victor in America</t>
+          <t>Victor in Amerika</t>
         </is>
       </c>
       <c r="C117" t="inlineStr">
@@ -4107,7 +4107,7 @@
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>With Marine Le Pen, a right-wing populist takes over the leadership of the parliamentary group</t>
+          <t>Mit Marine Le Pen übernimmt eine Rechtspopulistin die Fraktionsführung</t>
         </is>
       </c>
       <c r="C118" t="inlineStr">
@@ -4138,7 +4138,7 @@
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>Energy policy: Hydrogen is questionable as a climate-friendly energy source</t>
+          <t>Energiepolitik: Wasserstoff ist als klimafreundlicher Energieträger fragwürdig</t>
         </is>
       </c>
       <c r="C119" t="inlineStr">
@@ -4169,7 +4169,7 @@
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>Religious leaders say Covid vaccinations are to blame for rise in “demonic possession”.</t>
+          <t>Religiöse Führer sagen, dass Covid-Impfungen für den Anstieg von „dämonischen Besessenheit“ verantwortlich ist</t>
         </is>
       </c>
       <c r="C120" t="inlineStr">
@@ -4200,7 +4200,7 @@
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>WHO vaccination campaign with fatal consequences: More and more cases of “vaccine polio” in Africa</t>
+          <t>WHO-Impfkampagne mit fatalen Folgen: Immer mehr Fälle von „Impf-Polio” in Afrika</t>
         </is>
       </c>
       <c r="C121" t="inlineStr">
@@ -4231,7 +4231,7 @@
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>Climate change: How “Spiegel” calls for left-wing violence</t>
+          <t>Klimawandel: Wie der „Spiegel“ zu linker Gewalt aufruft</t>
         </is>
       </c>
       <c r="C122" t="inlineStr">
@@ -4262,7 +4262,7 @@
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>“There is no gas. It is a government invention” – Querheizer looks forward to winter in a relaxed manner</t>
+          <t>"Gas gibt es gar nicht. Es ist eine Erfindung der Regierung" – Querheizer sieht Winter entspannt entgegen</t>
         </is>
       </c>
       <c r="C123" t="inlineStr">
@@ -4293,7 +4293,7 @@
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>Mask or not? Be like Cem, Justin, Markus and Co!</t>
+          <t>Maske oder nicht? Sei wie Cem, Justin, Markus und Co!</t>
         </is>
       </c>
       <c r="C124" t="inlineStr">
@@ -4324,7 +4324,7 @@
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>NATO alone at home</t>
+          <t>Die Nato allein zuhaus</t>
         </is>
       </c>
       <c r="C125" t="inlineStr">
@@ -4355,7 +4355,7 @@
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>Anyone who wants to make archaic traditions part of our everyday life has to leave Germany!</t>
+          <t>Wer archaische Traditionen zu unserem Alltag machen will, hat Deutschland zu verlassen!</t>
         </is>
       </c>
       <c r="C126" t="inlineStr">
@@ -4386,7 +4386,7 @@
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>Putin's work and Kirill's contribution</t>
+          <t>Putins Werk und Kyrills Beitrag</t>
         </is>
       </c>
       <c r="C127" t="inlineStr">
@@ -4417,7 +4417,7 @@
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>A new church, a new faith, a new people</t>
+          <t>Eine neue Kirche, ein neuer Glauben, ein neues Volk</t>
         </is>
       </c>
       <c r="C128" t="inlineStr">
@@ -4448,7 +4448,7 @@
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>Prudery instead of pride</t>
+          <t>Prüderie statt Pride</t>
         </is>
       </c>
       <c r="C129" t="inlineStr">
@@ -4479,7 +4479,7 @@
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>Davos: “Climate protectors” fly in with 1,500 (!) private jets</t>
+          <t>Davos: „Klima-Schützer“ fliegen mit 1.500 (!) Privatjets ein</t>
         </is>
       </c>
       <c r="C130" t="inlineStr">
@@ -4510,7 +4510,7 @@
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>Global health governance is one of the fundamental elements of the New World Order and as such must be rejected and fought.</t>
+          <t>Global Health Governance ist eines der grundlegenden Elemente der Neuen Weltordnung und muss als solches abgelehnt und bekämpft werden.</t>
         </is>
       </c>
       <c r="C131" t="inlineStr">
@@ -4541,7 +4541,7 @@
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>The world's largest sponsors of their own imperial power are calling for the "decolonization" of Russia</t>
+          <t>Die weltweit größten Sponsoren eigener imperialer Macht fordern die "Dekolonisierung" Russlands</t>
         </is>
       </c>
       <c r="C132" t="inlineStr">
@@ -4572,7 +4572,7 @@
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>Redistribution, yes, but transparently</t>
+          <t>Umverteilung ja, aber transparent</t>
         </is>
       </c>
       <c r="C133" t="inlineStr">
@@ -4603,7 +4603,7 @@
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>A failed growth model</t>
+          <t>Ein gescheitertes Wachstumsmodell</t>
         </is>
       </c>
       <c r="C134" t="inlineStr">
@@ -4634,7 +4634,7 @@
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>Stop the masochism exercises: open Nordstream II!</t>
+          <t>Schluss mit den Masochismus-Übungen: Macht Nordstream II auf!</t>
         </is>
       </c>
       <c r="C135" t="inlineStr">
@@ -4665,7 +4665,7 @@
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>“CO₂ compensation does not solve the problem”</t>
+          <t>"CO₂-Kompensieren löst das Problem nicht"</t>
         </is>
       </c>
       <c r="C136" t="inlineStr">
@@ -4696,7 +4696,7 @@
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>What Europeans really think about migration and immigration</t>
+          <t>Was die Europäer über Migration und Einwanderung wirklich denken</t>
         </is>
       </c>
       <c r="C137" t="inlineStr">
@@ -4727,7 +4727,7 @@
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>But science is not dogma</t>
+          <t>Aber Wissenschaft ist kein Dogma</t>
         </is>
       </c>
       <c r="C138" t="inlineStr">
@@ -4758,7 +4758,7 @@
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>“Radical chic environmentalists”: Rampini criticizes the Greeks and De Gregorio gets irritated (Video)</t>
+          <t>„Radikale schicke Umweltschützer“: Rampini kritisiert die Griechen und De Gregorio ist irritiert (Video)</t>
         </is>
       </c>
       <c r="C139" t="inlineStr">
@@ -4789,7 +4789,7 @@
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>G7 in Munich: they matter so little that even the protesters no longer care</t>
+          <t>G7 in München: Sie sind so unbedeutend, dass selbst die Demonstranten sich nicht mehr darum kümmern</t>
         </is>
       </c>
       <c r="C140" t="inlineStr">
@@ -4820,7 +4820,7 @@
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>It's the usual Berlusconi: "Forza Italia at 20%, we will choose the prime minister". On defectors: "They will disappear like Alfano"</t>
+          <t>Es ist das übliche Berlusconi: „Forza Italia bei 20 %, wir werden den Premierminister wählen.“ Über Überläufer: „Sie werden verschwinden wie Alfano“</t>
         </is>
       </c>
       <c r="C141" t="inlineStr">
@@ -4851,7 +4851,7 @@
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>Sustainable finance and EU Taxonomy: what changes?</t>
+          <t>Nachhaltiges Finanzwesen und EU-Taxonomie: Was ändert sich?</t>
         </is>
       </c>
       <c r="C142" t="inlineStr">
@@ -4882,7 +4882,7 @@
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>DRAGHI FALLS, PUTIN ENJOYS - GRAMELLINI: “SORRY FOR THE MALICIOUS THINKING (IT WILL BE THE HEAT), BUT CONSIDERING THE COMMON POSITION OF CONTE AND SALVINI ON THE WAR, THE TRUE MYSTERY IS NOT THAT THE GOVERNMENT HAS FALLEN, BUT HOW IT HAS MANAGED TO LAST UNTIL YESTERDAY…”</t>
+          <t>DRAGHI FÄLLT, PUTIN GENIEßT - GRAMELLINI: „ENTSCHULDIGUNG FÜR DAS BÖSSE DENKEN (ES WIRD DIE HITZE SEIN), ABER IN ANBETRACHT DER GEMEINSAMEN POSITION VON CONTE UND SALVINI ZUM KRIEG IST DAS WAHRE GEHEIMNIS NICHT, DASS DIE REGIERUNG GEFALLEN IST, SONDERN, WIE SIE ES GESCHAFFT HAT, BIS GESTERN DAUERZUHALTEN…“</t>
         </is>
       </c>
       <c r="C143" t="inlineStr">
@@ -4913,7 +4913,7 @@
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>The anti-Putin dilemma of the German greens: “How many minutes can the shower last?”</t>
+          <t>Das Anti-Putin-Dilemma der deutschen Grünen: „Wie viele Minuten kann der Schauer dauern?“</t>
         </is>
       </c>
       <c r="C144" t="inlineStr">
@@ -4944,7 +4944,7 @@
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>Brazil: no to sanctions on Russia, or there will be world hunger. The real economy beats the paper one</t>
+          <t>Brasilien: Nein zu Sanktionen gegen Russland, sonst gibt es Welthunger. Die Realwirtschaft übertrifft die Papierwirtschaft</t>
         </is>
       </c>
       <c r="C145" t="inlineStr">
@@ -4975,7 +4975,7 @@
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>The next alarms: hot autumn? No very cold</t>
+          <t>Die nächsten Alarme: heißer Herbst? Nein, sehr kalt</t>
         </is>
       </c>
       <c r="C146" t="inlineStr">
@@ -5006,7 +5006,7 @@
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>Covid and vaccine, Galli: the obligation remains for those over 50. No amnesty for anti-vaxers</t>
+          <t>Covid und Impfstoff, Galli: Die Pflicht bleibt für über 50-Jährige bestehen. Keine Amnestie für Impfgegner</t>
         </is>
       </c>
       <c r="C147" t="inlineStr">
@@ -5037,7 +5037,7 @@
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>Russia-Ukraine war: Bolsonaro's Brazil remains neutral. But the president is pro-Russian</t>
+          <t>Russland-Ukraine-Krieg: Bolsonaros Brasilien bleibt neutral. Aber der Präsident ist pro-russisch</t>
         </is>
       </c>
       <c r="C148" t="inlineStr">
@@ -5068,7 +5068,7 @@
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>Monkeypox? It is racist, it "discriminates against Africans": the WHO will change the name of the disease</t>
+          <t>Affenpocken? Es ist rassistisch, es „diskriminiert Afrikaner“: Die WHO wird den Namen der Krankheit ändern</t>
         </is>
       </c>
       <c r="C149" t="inlineStr">
@@ -5099,7 +5099,7 @@
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>Turkish Defense Minister: Russia had nothing to do with the bombing of Odessa</t>
+          <t>Türkischer Verteidigungsminister: Russland hatte nichts mit der Bombardierung von Odessa zu tun</t>
         </is>
       </c>
       <c r="C150" t="inlineStr">
@@ -5130,7 +5130,7 @@
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>Migrants, almost 11 thousand have already landed this year. Meloni: «Naval blockade is the only solution»</t>
+          <t>Fast 11.000 Migranten sind dieses Jahr bereits gelandet. Meloni: «Seeblockade ist die einzige Lösung»</t>
         </is>
       </c>
       <c r="C151" t="inlineStr">
@@ -5161,7 +5161,7 @@
       </c>
       <c r="B152" t="inlineStr">
         <is>
-          <t>“Let's save the planet together”: all we were missing was the preaching book by Greta and the Dalai Lama</t>
+          <t>„Lasst uns gemeinsam den Planeten retten“: Uns fehlte nur noch das Predigtbuch von Greta und dem Dalai Lama</t>
         </is>
       </c>
       <c r="C152" t="inlineStr">
@@ -5192,7 +5192,7 @@
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>According to Moscow, the USA could be behind Covid and monkeypox</t>
+          <t>Laut Moskau könnten die USA hinter Covid und den Affenpocken stecken</t>
         </is>
       </c>
       <c r="C153" t="inlineStr">
@@ -5223,7 +5223,7 @@
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t>UkrLeaks: Nazis for export, from the United States to Kiev</t>
+          <t>UkrLeaks: Nazis für den Export, von den USA nach Kiew</t>
         </is>
       </c>
       <c r="C154" t="inlineStr">
@@ -5254,7 +5254,7 @@
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t>Energy: IEA, first global crisis, accelerate the transition</t>
+          <t>Energie: IEA, erste globale Krise, beschleunigt den Übergang</t>
         </is>
       </c>
       <c r="C155" t="inlineStr">
@@ -5285,7 +5285,7 @@
       </c>
       <c r="B156" t="inlineStr">
         <is>
-          <t>Salvini attacks the Ius Scholae again: "True Italians are illiterate"</t>
+          <t>Salvini greift das Ius Scholae erneut an: „Echte Italiener sind Analphabeten“</t>
         </is>
       </c>
       <c r="C156" t="inlineStr">
@@ -5316,7 +5316,7 @@
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t>Engaging BoomersThe climate movement cannot remain just a story of kids</t>
+          <t>Boomer einbinden Die Klimabewegung darf nicht nur eine Kindergeschichte bleiben</t>
         </is>
       </c>
       <c r="C157" t="inlineStr">
@@ -5347,7 +5347,7 @@
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>The UN asks Kiev, Moscow, the USA and the EU to respect the agreements on Russian and Ukrainian wheat</t>
+          <t>Die UN fordern Kiew, Moskau, die USA und die EU auf, die Abkommen über russischen und ukrainischen Weizen einzuhalten</t>
         </is>
       </c>
       <c r="C158" t="inlineStr">
@@ -5378,7 +5378,7 @@
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>The break is over</t>
+          <t>Die Pause ist vorbei</t>
         </is>
       </c>
       <c r="C159" t="inlineStr">
@@ -5409,7 +5409,7 @@
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>“Monkeypox has changed in a surprising way”</t>
+          <t>„Affenpocken haben sich auf überraschende Weise verändert“</t>
         </is>
       </c>
       <c r="C160" t="inlineStr">
@@ -5440,7 +5440,7 @@
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t>If voting served any purpose, the Anti-Vax people wouldn't let it.</t>
+          <t>Wenn die Abstimmung irgendeinen Zweck hätte, würden die Anti-Vax-Leute es nicht zulassen.</t>
         </is>
       </c>
       <c r="C161" t="inlineStr">
@@ -5471,7 +5471,7 @@
       </c>
       <c r="B162" t="inlineStr">
         <is>
-          <t>The physicist Prodi against Gretinism: "But like CO2, global warming obeys natural cycles"</t>
+          <t>Der Physiker Prodi gegen den Gretinismus: „Aber wie CO2 folgt auch die globale Erwärmung natürlichen Kreisläufen“</t>
         </is>
       </c>
       <c r="C162" t="inlineStr">
@@ -5502,7 +5502,7 @@
       </c>
       <c r="B163" t="inlineStr">
         <is>
-          <t>Pay attention to the French lesson. He can also teach Italy something</t>
+          <t>Achten Sie auf die Französischlektion. Er kann Italien auch etwas beibringen</t>
         </is>
       </c>
       <c r="C163" t="inlineStr">
@@ -5533,7 +5533,7 @@
       </c>
       <c r="B164" t="inlineStr">
         <is>
-          <t>Super environmentalist Germany forced to return to coal.</t>
+          <t>Super-Umweltschützer Deutschland gezwungen, zur Kohle zurückzukehren.</t>
         </is>
       </c>
       <c r="C164" t="inlineStr">
@@ -5564,7 +5564,7 @@
       </c>
       <c r="B165" t="inlineStr">
         <is>
-          <t>The “price” Russia must pay for using military force</t>
+          <t>Der „Preis“, den Russland für den Einsatz militärischer Gewalt zahlen muss</t>
         </is>
       </c>
       <c r="C165" t="inlineStr">
@@ -5595,7 +5595,7 @@
       </c>
       <c r="B166" t="inlineStr">
         <is>
-          <t>TO THE VOTE! TO THE VOTE! THE SPEAKING POLITICIANS</t>
+          <t>ZUR ABSTIMME! ZUR ABSTIMME! DIE SPRECHENDEN POLITIKER</t>
         </is>
       </c>
       <c r="C166" t="inlineStr">
@@ -5626,7 +5626,7 @@
       </c>
       <c r="B167" t="inlineStr">
         <is>
-          <t>Ukraine effectNow Iceland is also tempted to join the EU</t>
+          <t>Ukraine-EffektJetzt ist auch Island versucht, der EU beizutreten</t>
         </is>
       </c>
       <c r="C167" t="inlineStr">
@@ -5657,7 +5657,7 @@
       </c>
       <c r="B168" t="inlineStr">
         <is>
-          <t>The United States is extending its tentacles towards Russia and China through the uprisings in Central Asia</t>
+          <t>Durch die Aufstände in Zentralasien strecken die Vereinigten Staaten ihre Tentakel Richtung Russland und China aus</t>
         </is>
       </c>
       <c r="C168" t="inlineStr">
@@ -5688,7 +5688,7 @@
       </c>
       <c r="B169" t="inlineStr">
         <is>
-          <t>Coronavirus, Bolsonaro: "Many people die in Italy because it is a country of old people"</t>
+          <t>Coronavirus, Bolsonaro: „In Italien sterben viele Menschen, weil es ein Land der alten Menschen ist“</t>
         </is>
       </c>
       <c r="C169" t="inlineStr">
@@ -5719,7 +5719,7 @@
       </c>
       <c r="B170" t="inlineStr">
         <is>
-          <t>Italy uses "humanitarian corridors" to import migrants from Greece</t>
+          <t>Italien nutzt „humanitäre Korridore“, um Migranten aus Griechenland zu importieren</t>
         </is>
       </c>
       <c r="C170" t="inlineStr">
@@ -5750,7 +5750,7 @@
       </c>
       <c r="B171" t="inlineStr">
         <is>
-          <t>Migrants, the silent invasion: another 573 landed in Augusta. But Lamorgese doesn't lift a finger</t>
+          <t>Migranten, die stille Invasion: Weitere 573 landeten in Augusta. Doch Lamorgese rührt keinen Finger</t>
         </is>
       </c>
       <c r="C171" t="inlineStr">
@@ -5781,7 +5781,7 @@
       </c>
       <c r="B172" t="inlineStr">
         <is>
-          <t>Erich Vad, Merkel's former advisor: "USA and London can drag us into World War III"</t>
+          <t>Erich Vad, Merkels ehemaliger Berater: „USA und London können uns in den Dritten Weltkrieg hineinziehen“</t>
         </is>
       </c>
       <c r="C172" t="inlineStr">
@@ -5812,7 +5812,7 @@
       </c>
       <c r="B173" t="inlineStr">
         <is>
-          <t>1 - TRUMP'S RALLY FOR THE ALASKA ELECTIONS: "WITH THE GREENHOUSE EFFECT MORE SEA VIEW HOUSES"</t>
+          <t>1 – Trumps Kundgebung für die Wahlen in Alaska: „Mit Treibhauseffekt mehr Häuser mit Meerblick“</t>
         </is>
       </c>
       <c r="C173" t="inlineStr">
@@ -5843,7 +5843,7 @@
       </c>
       <c r="B174" t="inlineStr">
         <is>
-          <t>CLIMATE: GLOBAL WARMING will last a LONG time and the first victim could be MAN. A STUDY reveals it</t>
+          <t>KLIMA: Die globale Erwärmung wird noch LANGE anhalten und das erste Opfer könnte der Mensch sein. Eine Studie verrät es</t>
         </is>
       </c>
       <c r="C174" t="inlineStr">
@@ -5874,7 +5874,7 @@
       </c>
       <c r="B175" t="inlineStr">
         <is>
-          <t>“The Great Game” II: British activity in Ukraine</t>
+          <t>„The Great Game“ II: Britische Aktivitäten in der Ukraine</t>
         </is>
       </c>
       <c r="C175" t="inlineStr">
@@ -5905,7 +5905,7 @@
       </c>
       <c r="B176" t="inlineStr">
         <is>
-          <t>Germany, Economy Minister Habeck: "We face the biggest gas crisis"</t>
+          <t>Deutschland, Wirtschaftsminister Habeck: „Wir stehen vor der größten Gaskrise“</t>
         </is>
       </c>
       <c r="C176" t="inlineStr">
@@ -5936,7 +5936,7 @@
       </c>
       <c r="B177" t="inlineStr">
         <is>
-          <t>Ecr, Fitto: EU-NATO cooperate more and more to guarantee the choice of countries to join the alliance</t>
+          <t>Ecr, Fitto: EU-NATO kooperieren immer mehr, um die Auswahl der Länder zu gewährleisten, die dem Bündnis beitreten möchten</t>
         </is>
       </c>
       <c r="C177" t="inlineStr">
@@ -5967,7 +5967,7 @@
       </c>
       <c r="B178" t="inlineStr">
         <is>
-          <t>Lampedusa hotspot collapsing, Pisano: "Useless taxi ships sent by the government, we are the only ones defending the Italian borders"</t>
+          <t>Hotspot Lampedusa kollabiert, Pisano: „Von der Regierung geschickte nutzlose Taxischiffe, wir sind die Einzigen, die die italienischen Grenzen verteidigen“</t>
         </is>
       </c>
       <c r="C178" t="inlineStr">
@@ -5998,7 +5998,7 @@
       </c>
       <c r="B179" t="inlineStr">
         <is>
-          <t>The "advice" of the EU Commission and IMF: the Troika returns to threaten Italy</t>
+          <t>Der „Rat“ von EU-Kommission und IWF: Die Troika kehrt zurück, um Italien zu bedrohen</t>
         </is>
       </c>
       <c r="C179" t="inlineStr">
@@ -6029,7 +6029,7 @@
       </c>
       <c r="B180" t="inlineStr">
         <is>
-          <t>US plan fails in Ukraine</t>
+          <t>US-Plan scheitert in der Ukraine</t>
         </is>
       </c>
       <c r="C180" t="inlineStr">
@@ -6060,7 +6060,7 @@
       </c>
       <c r="B181" t="inlineStr">
         <is>
-          <t>The “Insect Allies” program – DARPA's Pandora's Box</t>
+          <t>Das „Insect Allies“-Programm – die Büchse der Pandora der DARPA</t>
         </is>
       </c>
       <c r="C181" t="inlineStr">
@@ -6091,7 +6091,7 @@
       </c>
       <c r="B182" t="inlineStr">
         <is>
-          <t>Wuhan, welcome back lockdown: 1 million people locked up due to 4 asymptomatic cases</t>
+          <t>Wuhan, willkommener Lockdown: 1 Million Menschen wegen 4 asymptomatischen Fällen eingesperrt</t>
         </is>
       </c>
       <c r="C182" t="inlineStr">
@@ -6122,7 +6122,7 @@
       </c>
       <c r="B183" t="inlineStr">
         <is>
-          <t>in "Wiadomości" TVP! How Tusk and the Germans "invented mercury"</t>
+          <t>in „Wiadomości“ TVP! Wie Tusk und die Deutschen „Quecksilber erfanden“</t>
         </is>
       </c>
       <c r="C183" t="inlineStr">
@@ -6153,7 +6153,7 @@
       </c>
       <c r="B184" t="inlineStr">
         <is>
-          <t>Not Czarnek, not Najman, but Anna-Maria Żukowska. The Left MP won an unusual competition</t>
+          <t>Nicht Czarnek, nicht Najman, sondern Anna-Maria Żukowska. Der Linke-Abgeordnete gewann einen ungewöhnlichen Wettbewerb</t>
         </is>
       </c>
       <c r="C184" t="inlineStr">
@@ -6184,7 +6184,7 @@
       </c>
       <c r="B185" t="inlineStr">
         <is>
-          <t>Coronavirus. In Wuhan, there is another lockdown for millions of citizens. Four cases of infection were detected</t>
+          <t>Coronavirus. In Wuhan kommt es erneut zu einem Lockdown für Millionen Bürger. Es wurden vier Infektionsfälle festgestellt</t>
         </is>
       </c>
       <c r="C185" t="inlineStr">
@@ -6215,7 +6215,7 @@
       </c>
       <c r="B186" t="inlineStr">
         <is>
-          <t>The Great Barrier Reef is great in more than just name. She just stood up to climate change</t>
+          <t>Das Great Barrier Reef ist nicht nur wegen seines Namens großartig. Sie hat dem Klimawandel einfach die Stirn geboten</t>
         </is>
       </c>
       <c r="C186" t="inlineStr">
@@ -6246,7 +6246,7 @@
       </c>
       <c r="B187" t="inlineStr">
         <is>
-          <t>Sylwia Spurek: What gives us the right to exploit a dairy cow?</t>
+          <t>Sylwia Spurek: Was gibt uns das Recht, eine Milchkuh auszubeuten?</t>
         </is>
       </c>
       <c r="C187" t="inlineStr">
@@ -6277,7 +6277,7 @@
       </c>
       <c r="B188" t="inlineStr">
         <is>
-          <t>DIFFERENT FRONTS OF ONE WAR</t>
+          <t>VERSCHIEDENE FRONTEN EINES KRIEGES</t>
         </is>
       </c>
       <c r="C188" t="inlineStr">
@@ -6308,7 +6308,7 @@
       </c>
       <c r="B189" t="inlineStr">
         <is>
-          <t>The number of coronavirus infections in Poland is still not decreasing. New report of the Ministry of Health</t>
+          <t>Die Zahl der Coronavirus-Infektionen in Polen geht weiterhin nicht zurück. Neuer Bericht des Gesundheitsministeriums</t>
         </is>
       </c>
       <c r="C189" t="inlineStr">
@@ -6339,7 +6339,7 @@
       </c>
       <c r="B190" t="inlineStr">
         <is>
-          <t>Most Poles do not want the return of coronavirus restrictions, but PiS voters do</t>
+          <t>Die meisten Polen wollen die Rückkehr der Corona-Beschränkungen nicht, die PiS-Wähler hingegen schon</t>
         </is>
       </c>
       <c r="C190" t="inlineStr">
@@ -6370,7 +6370,7 @@
       </c>
       <c r="B191" t="inlineStr">
         <is>
-          <t>Anger towards Germany is rising in Poland. "Too Little, Too Late"</t>
+          <t>In Polen wächst die Wut auf Deutschland. „Zu wenig, zu spät“</t>
         </is>
       </c>
       <c r="C191" t="inlineStr">
@@ -6401,7 +6401,7 @@
       </c>
       <c r="B192" t="inlineStr">
         <is>
-          <t>Polish excavation</t>
+          <t>Polnische Ausgrabung</t>
         </is>
       </c>
       <c r="C192" t="inlineStr">
@@ -6432,7 +6432,7 @@
       </c>
       <c r="B193" t="inlineStr">
         <is>
-          <t>A controversial opinion of a German politician. "Not only Russia, but also the USA is evil"</t>
+          <t>Eine kontroverse Meinung eines deutschen Politikers. „Nicht nur Russland, auch die USA sind böse“</t>
         </is>
       </c>
       <c r="C193" t="inlineStr">
@@ -6463,7 +6463,7 @@
       </c>
       <c r="B194" t="inlineStr">
         <is>
-          <t>Western sanctions are working. The Russian economy is bleeding</t>
+          <t>Die Sanktionen des Westens wirken. Die russische Wirtschaft blutet</t>
         </is>
       </c>
       <c r="C194" t="inlineStr">
@@ -6494,7 +6494,7 @@
       </c>
       <c r="B195" t="inlineStr">
         <is>
-          <t>EU. However, Tusk received an "order for Poland"</t>
+          <t>EU. Tusk erhielt jedoch einen „Befehl für Polen“</t>
         </is>
       </c>
       <c r="C195" t="inlineStr">
@@ -6525,7 +6525,7 @@
       </c>
       <c r="B196" t="inlineStr">
         <is>
-          <t>Ziobro on Covid certificates: I am not a supporter</t>
+          <t>Ziobro zu Covid-Zertifikaten: Ich bin kein Unterstützer</t>
         </is>
       </c>
       <c r="C196" t="inlineStr">
@@ -6556,7 +6556,7 @@
       </c>
       <c r="B197" t="inlineStr">
         <is>
-          <t>Andrzej Duda ignores the devastating climate report. Her thoughts are at Antek Królikowski's wedding</t>
+          <t>Andrzej Duda ignoriert den verheerenden Klimabericht. Ihre Gedanken sind bei Antek Królikowskis Hochzeit</t>
         </is>
       </c>
       <c r="C197" t="inlineStr">
@@ -6587,7 +6587,7 @@
       </c>
       <c r="B198" t="inlineStr">
         <is>
-          <t>Speaker of the Duma: The arsenal of Western sanctions has been exhausted. Russia can benefit</t>
+          <t>Duma-Sprecher: Das Arsenal westlicher Sanktionen ist erschöpft. Russland kann profitieren</t>
         </is>
       </c>
       <c r="C198" t="inlineStr">
@@ -6618,7 +6618,7 @@
       </c>
       <c r="B199" t="inlineStr">
         <is>
-          <t>Greta Thunberg. An atmospheric symbol without meaning [COMMENT]</t>
+          <t>Greta Thunberg. Ein atmosphärisches Symbol ohne Bedeutung [KOMMENTAR]</t>
         </is>
       </c>
       <c r="C199" t="inlineStr">
@@ -6649,7 +6649,7 @@
       </c>
       <c r="B200" t="inlineStr">
         <is>
-          <t>LEGAL ABORTION. "IN THIS VOTING THE CHOICE WAS VERY SIMPLE, YOU ARE EITHER FOR WOMEN OR AGAINST THEM"</t>
+          <t>Legale Abtreibung. „Bei dieser Abstimmung war die Wahl sehr einfach, Sie sind entweder für Frauen oder dagegen.“</t>
         </is>
       </c>
       <c r="C200" t="inlineStr">
@@ -6680,7 +6680,7 @@
       </c>
       <c r="B201" t="inlineStr">
         <is>
-          <t>In Italy, the far right is politicizing anti-vaxxers</t>
+          <t>In Italien politisiert die extreme Rechte Impfgegner</t>
         </is>
       </c>
       <c r="C201" t="inlineStr">
@@ -6711,7 +6711,7 @@
       </c>
       <c r="B202" t="inlineStr">
         <is>
-          <t>Niedzielski: The infectiousness of monkeypox is not high</t>
+          <t>Niedzielski: Die Ansteckungsgefahr von Affenpocken ist nicht hoch</t>
         </is>
       </c>
       <c r="C202" t="inlineStr">
@@ -6742,7 +6742,7 @@
       </c>
       <c r="B203" t="inlineStr">
         <is>
-          <t>Wolski: For the Russians, using cluster bombs is like going out for bread</t>
+          <t>Wolski: Für die Russen ist der Einsatz von Streubomben wie ein Brotholen</t>
         </is>
       </c>
       <c r="C203" t="inlineStr">
@@ -6773,7 +6773,7 @@
       </c>
       <c r="B204" t="inlineStr">
         <is>
-          <t>"Hypocrisy". Macron under fire after revealing vacation photos</t>
+          <t>"Heuchelei". Macron steht unter Beschuss, nachdem er Urlaubsfotos enthüllt hat</t>
         </is>
       </c>
       <c r="C204" t="inlineStr">
@@ -6804,7 +6804,7 @@
       </c>
       <c r="B205" t="inlineStr">
         <is>
-          <t>"Zelensky's industry" is silent about the war. Ukraine resents satirists from Russia for not condemning Putin</t>
+          <t>„Selenskys Industrie“ schweigt über den Krieg. Die Ukraine nimmt es Satirikern aus Russland übel, weil sie Putin nicht verurteilen</t>
         </is>
       </c>
       <c r="C205" t="inlineStr">
@@ -6835,7 +6835,7 @@
       </c>
       <c r="B206" t="inlineStr">
         <is>
-          <t>Colonialism is still going on. And it is one of the causes of climate change</t>
+          <t>Der Kolonialismus ist immer noch im Gange. Und es ist eine der Ursachen des Klimawandels</t>
         </is>
       </c>
       <c r="C206" t="inlineStr">
@@ -6866,7 +6866,7 @@
       </c>
       <c r="B207" t="inlineStr">
         <is>
-          <t>In South Africa, they have already turned off the lights</t>
+          <t>In Südafrika haben sie bereits das Licht ausgeschaltet</t>
         </is>
       </c>
       <c r="C207" t="inlineStr">
@@ -6897,7 +6897,7 @@
       </c>
       <c r="B208" t="inlineStr">
         <is>
-          <t>Nord Stream 2 is the biggest problem in German politics</t>
+          <t>Nord Stream 2 ist das größte Problem der deutschen Politik</t>
         </is>
       </c>
       <c r="C208" t="inlineStr">
@@ -6928,7 +6928,7 @@
       </c>
       <c r="B209" t="inlineStr">
         <is>
-          <t>Kim Jong Un wants to support Putin's army. This is what equipment North Korea has.</t>
+          <t>Kim Jong Un will Putins Armee unterstützen. Über diese Ausrüstung verfügt Nordkorea.</t>
         </is>
       </c>
       <c r="C209" t="inlineStr">
@@ -6959,7 +6959,7 @@
       </c>
       <c r="B210" t="inlineStr">
         <is>
-          <t>Is another wave of restrictions coming?</t>
+          <t>Kommt eine weitere Welle von Beschränkungen?</t>
         </is>
       </c>
       <c r="C210" t="inlineStr">
@@ -6990,7 +6990,7 @@
       </c>
       <c r="B211" t="inlineStr">
         <is>
-          <t>Over a hundred coronavirus infections linked to one bar. "Dangerous wave" in Beijing</t>
+          <t>Über hundert Coronavirus-Infektionen im Zusammenhang mit einem Riegel. „Gefährliche Welle“ in Peking</t>
         </is>
       </c>
       <c r="C211" t="inlineStr">

</xml_diff>